<commit_message>
Insere resultados com rag_1
</commit_message>
<xml_diff>
--- a/Resultados consolidados.xlsx
+++ b/Resultados consolidados.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\P_8454\Desktop\rag_legislacao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caris\Desktop\rag_legislacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE6B313-24E5-4D24-B0BF-A6BE64B68022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11415"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
   <si>
     <t>Sem contexto</t>
   </si>
@@ -44,19 +45,28 @@
     <t>Sabia-4</t>
   </si>
   <si>
-    <t>RAG_5 - apenas artigos sem histórico</t>
-  </si>
-  <si>
-    <t>RAG_5 - apenas artigos com histórico</t>
-  </si>
-  <si>
-    <t>RAG_5 - hierárquicos</t>
+    <t>RAG 5</t>
+  </si>
+  <si>
+    <t>apenas artigos sem histórico</t>
+  </si>
+  <si>
+    <t>apenas artigos com histórico</t>
+  </si>
+  <si>
+    <t>hierárquicos</t>
+  </si>
+  <si>
+    <t>RAG 1</t>
+  </si>
+  <si>
+    <t>RAG 10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -74,7 +84,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -87,8 +97,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -107,11 +123,51 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -120,7 +176,30 @@
     <xf numFmtId="10" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -402,112 +481,241 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C5:H9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="C5:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="40.7109375" customWidth="1"/>
     <col min="4" max="8" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:8" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
+    <row r="5" spans="3:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="7"/>
+      <c r="D5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="3:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="1" t="s">
+    <row r="6" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="8"/>
+      <c r="D6" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+    </row>
+    <row r="7" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="10"/>
+      <c r="D7" s="13">
         <v>0.48770000000000002</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E7" s="13">
         <v>0.64710000000000001</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F7" s="13">
         <v>0.73060000000000003</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G7" s="13">
         <v>0.63759999999999994</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H7" s="13">
         <v>0.67359999999999998</v>
       </c>
     </row>
-    <row r="7" spans="3:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="1" t="s">
+    <row r="8" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="14"/>
+      <c r="D8" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+    </row>
+    <row r="9" spans="3:8" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="12">
+        <v>0.55979999999999996</v>
+      </c>
+      <c r="E9" s="12">
+        <v>0.70020000000000004</v>
+      </c>
+      <c r="F9" s="12">
+        <v>0.78369999999999995</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="12">
+        <v>0.72489999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.5655</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.69640000000000002</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0.78369999999999995</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2">
+        <v>0.71540000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="3:8" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="11">
+        <v>0.54649999999999999</v>
+      </c>
+      <c r="E11" s="11">
+        <v>0.67930000000000001</v>
+      </c>
+      <c r="F11" s="11">
+        <v>0.76849999999999996</v>
+      </c>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11">
+        <v>0.71540000000000004</v>
+      </c>
+    </row>
+    <row r="12" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="14"/>
+      <c r="D12" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="3">
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+    </row>
+    <row r="13" spans="3:8" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="3">
         <v>0.57310000000000005</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E13" s="2">
         <v>0.70589999999999997</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F13" s="2">
         <v>0.79890000000000005</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G13" s="2">
         <v>0.65839999999999999</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H13" s="2">
         <v>0.73809999999999998</v>
       </c>
     </row>
-    <row r="8" spans="3:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="1" t="s">
+    <row r="14" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.55030000000000001</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0.7097</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0.80269999999999997</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0.66410000000000002</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0.74570000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="3:8" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.54079999999999995</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.71919999999999995</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0.81399999999999995</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0.6603</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0.74760000000000004</v>
+      </c>
+    </row>
+    <row r="16" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="14"/>
+      <c r="D16" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+    </row>
+    <row r="17" spans="3:8" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="4">
-        <v>0.55030000000000001</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0.7097</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0.80269999999999997</v>
-      </c>
-      <c r="G8" s="3">
-        <v>0.66410000000000002</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0.74570000000000003</v>
-      </c>
-    </row>
-    <row r="9" spans="3:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="1" t="s">
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="2">
-        <v>0.54079999999999995</v>
-      </c>
-      <c r="E9" s="3">
-        <v>0.71919999999999995</v>
-      </c>
-      <c r="F9" s="3">
-        <v>0.81399999999999995</v>
-      </c>
-      <c r="G9" s="2">
-        <v>0.6603</v>
-      </c>
-      <c r="H9" s="3">
-        <v>0.74760000000000004</v>
-      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D16:H16"/>
+  </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Adicionado experimentos com gpt-5.4 nano e mini para 10 chunks
</commit_message>
<xml_diff>
--- a/Resultados consolidados.xlsx
+++ b/Resultados consolidados.xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caris\Desktop\rag_legislacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE6B313-24E5-4D24-B0BF-A6BE64B68022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E0FAD6-586C-482E-9C49-3F67A548A1AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -176,7 +187,7 @@
     <xf numFmtId="10" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -185,23 +196,23 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,14 +493,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C5:H19"/>
+  <dimension ref="C5:N19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="40.7109375" customWidth="1"/>
     <col min="4" max="8" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="3:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C5" s="7"/>
       <c r="D5" s="7" t="s">
         <v>1</v>
@@ -507,63 +518,62 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="8"/>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-    </row>
-    <row r="7" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="10"/>
-      <c r="D7" s="13">
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="11">
         <v>0.48770000000000002</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="11">
         <v>0.64710000000000001</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="11">
         <v>0.73060000000000003</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="11">
         <v>0.63759999999999994</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="11">
         <v>0.67359999999999998</v>
       </c>
     </row>
-    <row r="8" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C8" s="14"/>
-      <c r="D8" s="15" t="s">
+    <row r="8" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="12"/>
+      <c r="D8" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-    </row>
-    <row r="9" spans="3:8" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+    </row>
+    <row r="9" spans="3:14" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="10">
         <v>0.55979999999999996</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="10">
         <v>0.70020000000000004</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="10">
         <v>0.78369999999999995</v>
       </c>
       <c r="G9" s="6"/>
-      <c r="H9" s="12">
+      <c r="H9" s="10">
         <v>0.72489999999999999</v>
       </c>
     </row>
-    <row r="10" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
         <v>8</v>
       </c>
@@ -581,35 +591,35 @@
         <v>0.71540000000000004</v>
       </c>
     </row>
-    <row r="11" spans="3:8" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:14" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="9">
         <v>0.54649999999999999</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="9">
         <v>0.67930000000000001</v>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="9">
         <v>0.76849999999999996</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11">
+      <c r="G11" s="9"/>
+      <c r="H11" s="9">
         <v>0.71540000000000004</v>
       </c>
     </row>
-    <row r="12" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="14"/>
-      <c r="D12" s="15" t="s">
+    <row r="12" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="12"/>
+      <c r="D12" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-    </row>
-    <row r="13" spans="3:8" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+    </row>
+    <row r="13" spans="3:14" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
         <v>7</v>
       </c>
@@ -628,8 +638,14 @@
       <c r="H13" s="2">
         <v>0.73809999999999998</v>
       </c>
-    </row>
-    <row r="14" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
+      <c r="N13" s="15"/>
+    </row>
+    <row r="14" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="s">
         <v>8</v>
       </c>
@@ -648,8 +664,14 @@
       <c r="H14" s="2">
         <v>0.74570000000000003</v>
       </c>
-    </row>
-    <row r="15" spans="3:8" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+    </row>
+    <row r="15" spans="3:14" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
         <v>9</v>
       </c>
@@ -668,46 +690,82 @@
       <c r="H15" s="3">
         <v>0.74760000000000004</v>
       </c>
-    </row>
-    <row r="16" spans="3:8" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="14"/>
-      <c r="D16" s="15" t="s">
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="15"/>
+    </row>
+    <row r="16" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="12"/>
+      <c r="D16" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-    </row>
-    <row r="17" spans="3:8" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+    </row>
+    <row r="17" spans="3:14" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="D17" s="10">
+        <v>0.56169999999999998</v>
+      </c>
+      <c r="E17" s="10">
+        <v>0.71350000000000002</v>
+      </c>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+    </row>
+    <row r="18" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
+      <c r="D18" s="4">
+        <v>0.55979999999999996</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0.70589999999999997</v>
+      </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
-    </row>
-    <row r="19" spans="3:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+    </row>
+    <row r="19" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
+      <c r="D19" s="4">
+        <v>0.55220000000000002</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0.70209999999999995</v>
+      </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
inserido resultados do rag_1 com o sabiazinho
</commit_message>
<xml_diff>
--- a/Resultados consolidados.xlsx
+++ b/Resultados consolidados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caris\Desktop\rag_legislacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E0FAD6-586C-482E-9C49-3F67A548A1AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1B0129-247F-4D6F-9871-2F2D493756E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -206,13 +206,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,13 +520,13 @@
     </row>
     <row r="6" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="8"/>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D7" s="11">
@@ -547,13 +547,13 @@
     </row>
     <row r="8" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="12"/>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
     </row>
     <row r="9" spans="3:14" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C9" s="5" t="s">
@@ -568,7 +568,9 @@
       <c r="F9" s="10">
         <v>0.78369999999999995</v>
       </c>
-      <c r="G9" s="6"/>
+      <c r="G9" s="6">
+        <v>0.65459999999999996</v>
+      </c>
       <c r="H9" s="10">
         <v>0.72489999999999999</v>
       </c>
@@ -586,7 +588,9 @@
       <c r="F10" s="3">
         <v>0.78369999999999995</v>
       </c>
-      <c r="G10" s="2"/>
+      <c r="G10" s="3">
+        <v>0.65839999999999999</v>
+      </c>
       <c r="H10" s="2">
         <v>0.71540000000000004</v>
       </c>
@@ -604,20 +608,22 @@
       <c r="F11" s="9">
         <v>0.76849999999999996</v>
       </c>
-      <c r="G11" s="9"/>
+      <c r="G11" s="9">
+        <v>0.64900000000000002</v>
+      </c>
       <c r="H11" s="9">
         <v>0.71540000000000004</v>
       </c>
     </row>
     <row r="12" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="12"/>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
     </row>
     <row r="13" spans="3:14" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
@@ -638,12 +644,12 @@
       <c r="H13" s="2">
         <v>0.73809999999999998</v>
       </c>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
-      <c r="N13" s="15"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="N13" s="13"/>
     </row>
     <row r="14" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="s">
@@ -664,12 +670,12 @@
       <c r="H14" s="2">
         <v>0.74570000000000003</v>
       </c>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
-      <c r="N14" s="15"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
     </row>
     <row r="15" spans="3:14" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
@@ -690,22 +696,22 @@
       <c r="H15" s="3">
         <v>0.74760000000000004</v>
       </c>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="15"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="13"/>
     </row>
     <row r="16" spans="3:14" ht="29.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C16" s="12"/>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
     </row>
     <row r="17" spans="3:14" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C17" s="1" t="s">
@@ -720,12 +726,12 @@
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15"/>
-      <c r="N17" s="15"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
     </row>
     <row r="18" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="1" t="s">
@@ -735,17 +741,17 @@
         <v>0.55979999999999996</v>
       </c>
       <c r="E18" s="4">
-        <v>0.70589999999999997</v>
+        <v>0.70779999999999998</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
     </row>
     <row r="19" spans="3:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="1" t="s">
@@ -760,12 +766,12 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="15"/>
-      <c r="M19" s="15"/>
-      <c r="N19" s="15"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>